<commit_message>
fixed an issue where start/end_date were not properly read
</commit_message>
<xml_diff>
--- a/exp_database/dummy_experiment/output/miappe_template_filled.xlsx
+++ b/exp_database/dummy_experiment/output/miappe_template_filled.xlsx
@@ -333,7 +333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1483,6 +1483,376 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/experiment/dummy_experiment_testtest</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>https://dummy_variety.ontology</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/scientific-object/so-dummy_plant_1/4</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>vocabulary:Plant</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>dummy_plant_1</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>['opensilex-sandbox:id/factor/dummy_experiment_testtest.water_stress.ww', 'opensilex-sandbox:id/factor/dummy_experiment_testtest.light_stress.wl']</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-08-12 16:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/experiment/dummy_experiment_testtest</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>https://dummy_variety.ontology</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/scientific-object/so-dummy_plant_2/4</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>vocabulary:Plant</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>dummy_plant_2</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>['opensilex-sandbox:id/factor/dummy_experiment_testtest.water_stress.ws', 'opensilex-sandbox:id/factor/dummy_experiment_testtest.light_stress.wl']</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-08-12 16:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/experiment/dummy_experiment_testtest</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>https://dummy_variety.ontology</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/scientific-object/so-dummy_plant_3/4</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>vocabulary:Plant</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>dummy_plant_3</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>['opensilex-sandbox:id/factor/dummy_experiment_testtest.water_stress.ws', 'opensilex-sandbox:id/factor/dummy_experiment_testtest.light_stress.ls']</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-08-12 16:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/experiment/dummy_experiment_testtest</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>https://dummy_variety.ontology</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/scientific-object/so-dummy_plant_4/4</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>vocabulary:Plant</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>dummy_plant_4</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>['opensilex-sandbox:id/factor/dummy_experiment_testtest.water_stress.ws', 'opensilex-sandbox:id/factor/dummy_experiment_testtest.light_stress.wl']</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-08-12 16:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/experiment/dummy_experiment_testtest</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>https://dummy_variety.ontology</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/scientific-object/so-dummy_plant_5/4</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>vocabulary:Plant</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>dummy_plant_5</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>['opensilex-sandbox:id/factor/dummy_experiment_testtest.water_stress.ww', 'opensilex-sandbox:id/factor/dummy_experiment_testtest.light_stress.wl']</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-08-12 16:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/experiment/dummy_experiment_testtest</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>https://dummy_variety.ontology</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/scientific-object/so-dummy_plant_6/4</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>vocabulary:Plant</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>dummy_plant_6</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>['opensilex-sandbox:id/factor/dummy_experiment_testtest.water_stress.ww', 'opensilex-sandbox:id/factor/dummy_experiment_testtest.light_stress.ls']</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-08-12 16:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/experiment/dummy_experiment_testtest</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>https://dummy_variety.ontology</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/scientific-object/so-dummy_plant_7/4</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>vocabulary:Plant</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>dummy_plant_7</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>['opensilex-sandbox:id/factor/dummy_experiment_testtest.water_stress.ww', 'opensilex-sandbox:id/factor/dummy_experiment_testtest.light_stress.wl']</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-08-12 16:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/experiment/dummy_experiment_testtest</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>https://dummy_variety.ontology</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/scientific-object/so-dummy_plant_8/4</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>vocabulary:Plant</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>dummy_plant_8</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>['opensilex-sandbox:id/factor/dummy_experiment_testtest.water_stress.ww', 'opensilex-sandbox:id/factor/dummy_experiment_testtest.light_stress.wl']</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-08-12 16:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/experiment/dummy_experiment_testtest</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>https://dummy_variety.ontology</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/scientific-object/so-dummy_plant_9/4</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>vocabulary:Plant</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>dummy_plant_9</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>['opensilex-sandbox:id/factor/dummy_experiment_testtest.water_stress.ww', 'opensilex-sandbox:id/factor/dummy_experiment_testtest.light_stress.ls']</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2026-08-12 16:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/experiment/dummy_experiment_testtest</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>https://dummy_variety.ontology</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/scientific-object/so-dummy_plant_10/4</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>vocabulary:Plant</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>dummy_plant_10</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>['opensilex-sandbox:id/factor/dummy_experiment_testtest.water_stress.ws', 'opensilex-sandbox:id/factor/dummy_experiment_testtest.light_stress.ls']</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-08-12 16:11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
updated the displayed gif
</commit_message>
<xml_diff>
--- a/exp_database/dummy_experiment/output/miappe_template_filled.xlsx
+++ b/exp_database/dummy_experiment/output/miappe_template_filled.xlsx
@@ -333,7 +333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2223,6 +2223,376 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/experiment/simple_github_presentation</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>https://dummy_variety.ontology</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/scientific-object/so-dummy_plant_1/6</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>vocabulary:Plant</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>dummy_plant_1</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>['opensilex-sandbox:id/factor/simple_github_presentation.water_stress.ww', 'opensilex-sandbox:id/factor/simple_github_presentation.light_stress.wl']</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2026-08-26 14:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/experiment/simple_github_presentation</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>https://dummy_variety.ontology</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/scientific-object/so-dummy_plant_2/6</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>vocabulary:Plant</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>dummy_plant_2</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>['opensilex-sandbox:id/factor/simple_github_presentation.water_stress.ws', 'opensilex-sandbox:id/factor/simple_github_presentation.light_stress.wl']</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-08-26 14:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/experiment/simple_github_presentation</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>https://dummy_variety.ontology</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/scientific-object/so-dummy_plant_3/6</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>vocabulary:Plant</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>dummy_plant_3</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>['opensilex-sandbox:id/factor/simple_github_presentation.water_stress.ws', 'opensilex-sandbox:id/factor/simple_github_presentation.light_stress.ls']</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026-08-26 14:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/experiment/simple_github_presentation</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>https://dummy_variety.ontology</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/scientific-object/so-dummy_plant_4/6</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>vocabulary:Plant</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>dummy_plant_4</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>['opensilex-sandbox:id/factor/simple_github_presentation.water_stress.ws', 'opensilex-sandbox:id/factor/simple_github_presentation.light_stress.wl']</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2026-08-26 14:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/experiment/simple_github_presentation</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>https://dummy_variety.ontology</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/scientific-object/so-dummy_plant_5/6</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>vocabulary:Plant</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>dummy_plant_5</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>['opensilex-sandbox:id/factor/simple_github_presentation.water_stress.ww', 'opensilex-sandbox:id/factor/simple_github_presentation.light_stress.wl']</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2026-08-26 14:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/experiment/simple_github_presentation</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>https://dummy_variety.ontology</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/scientific-object/so-dummy_plant_6/6</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>vocabulary:Plant</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>dummy_plant_6</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>['opensilex-sandbox:id/factor/simple_github_presentation.water_stress.ww', 'opensilex-sandbox:id/factor/simple_github_presentation.light_stress.ls']</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2026-08-26 14:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/experiment/simple_github_presentation</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>https://dummy_variety.ontology</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/scientific-object/so-dummy_plant_7/6</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>vocabulary:Plant</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>dummy_plant_7</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>['opensilex-sandbox:id/factor/simple_github_presentation.water_stress.ww', 'opensilex-sandbox:id/factor/simple_github_presentation.light_stress.wl']</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>2026-08-26 14:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/experiment/simple_github_presentation</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>https://dummy_variety.ontology</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/scientific-object/so-dummy_plant_8/6</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>vocabulary:Plant</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>dummy_plant_8</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>['opensilex-sandbox:id/factor/simple_github_presentation.water_stress.ww', 'opensilex-sandbox:id/factor/simple_github_presentation.light_stress.wl']</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2026-08-26 14:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/experiment/simple_github_presentation</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>https://dummy_variety.ontology</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/scientific-object/so-dummy_plant_9/6</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>vocabulary:Plant</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>dummy_plant_9</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>['opensilex-sandbox:id/factor/simple_github_presentation.water_stress.ww', 'opensilex-sandbox:id/factor/simple_github_presentation.light_stress.ls']</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2026-08-26 14:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/experiment/simple_github_presentation</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>https://dummy_variety.ontology</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>opensilex-sandbox:id/scientific-object/so-dummy_plant_10/6</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>vocabulary:Plant</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>dummy_plant_10</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>['opensilex-sandbox:id/factor/simple_github_presentation.water_stress.ws', 'opensilex-sandbox:id/factor/simple_github_presentation.light_stress.ls']</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2026-08-26 14:13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>